<commit_message>
user module Post operation done
</commit_message>
<xml_diff>
--- a/src/test/resources/Team01_RestAssured_Rebles_TestDataSheet.xlsx
+++ b/src/test/resources/Team01_RestAssured_Rebles_TestDataSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dineshdeshmukh/eclipse-workspace/Team01_RestAssured_Rebels/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAB675D8-5CD7-9C4D-B63C-E8B32E688F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2822732F-7638-4B46-951F-FB0ABF6696EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1300" windowWidth="38400" windowHeight="18900" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="1300" windowWidth="38400" windowHeight="18900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="52">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>Create_Valid_User_3</t>
-  </si>
-  <si>
-    <t>Create_User_Only_Mandatory_Fields</t>
   </si>
   <si>
     <t>/users/roleStatus</t>
@@ -232,6 +229,271 @@
     "status": "Active"
   }
 }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create_User_Empty_Payload </t>
+  </si>
+  <si>
+    <t>{
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_Frist_Name_Field</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName":   ,
+  "userLastName": "Mathur",
+  "userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": " ",
+  "userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_Last_Name_Field</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Patil",
+  "userMiddleName": "Desi",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "",
+  "userTimeZone": "EST",
+  "userLinkedinUrl": "www.linkedin.com",
+  "userEduUg": "BE",
+  "userEduPg": "PHD",
+  "userComments": "PASSED",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R02",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_Location</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R01",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_TimeZone</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_VisaStatus</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "",
+  "userRoleMaps": [
+    {
+      "roleId": "R01",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create_User_Empty_RoleId </t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H4",
+  "userRoleMaps": [
+    {
+      "roleId": "",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_RoleStatus</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H4",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": ""
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_LoginStatus</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H4",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create_User_Empty_Email </t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "&lt;random_phone&gt;",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H4",
+  "userRoleMaps": [
+    {
+      "roleId": "R03",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Empty_PhoneNumber</t>
+  </si>
+  <si>
+    <t>{
+  "userFirstName": "Sunny",
+  "userLastName": "Penny",
+  "userPhoneNumber": "",
+  "userLocation": "Atlanta",
+  "userTimeZone": "EST",
+  "userVisaStatus": "H1B",
+  "userRoleMaps": [
+    {
+      "roleId": "R01",
+      "userRoleStatus": "Active"
+    }
+  ],
+  "userLogin": {
+    "userLoginEmail": "&lt;random_email&gt;",
+    "loginStatus": "Active",
+    "status": "Active"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Create_User_Only_Mandatory_Field</t>
   </si>
 </sst>
 </file>
@@ -9882,7 +10144,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ECCC9A2-780E-422B-AA2C-B36256EC8A5E}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" style="11"/>
@@ -9909,7 +10171,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>20</v>
@@ -9923,7 +10185,7 @@
         <v>22</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>20</v>
@@ -9937,7 +10199,7 @@
         <v>23</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>20</v>
@@ -9948,16 +10210,170 @@
     </row>
     <row r="5" spans="1:4" ht="304" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" s="11">
         <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="380" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="380" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="380" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A10" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A11" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A12" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A13" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A14" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A15" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="11">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="11">
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>